<commit_message>
Add Candidates sheet to Hawaii café Excel
Update HI tracker with a second sheet of 8 additional Oahu candidates
(Cowrie, Cooke Street, Morning Glass, Aloha Matcha, Pua Blooms, Kai Coffee,
ARS Cafe, Dean & DeLuca) in the same tracker format.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX28XCL3v6f7LuJT98rxVZ
</commit_message>
<xml_diff>
--- a/07_markets/us/HI_cafe_priority_A.xlsx
+++ b/07_markets/us/HI_cafe_priority_A.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hawaii Priority A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hawaii Priority A'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priority A'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Candidates'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -573,7 +575,7 @@
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>抹茶・ほうじ茶に注力。美意識高く相性◎</t>
+          <t>抹茶・ほうじ茶に注力。相性◎</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -618,7 +620,7 @@
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>ハワイのコーヒー会社。ハンド点て抹茶＋自家シロップ・材料調達型</t>
+          <t>ハンド点て抹茶＋自家シロップ・材料調達型</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
@@ -663,7 +665,7 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>オーツミルクのボトルラテ。SNS強（12K）</t>
+          <t>オーツミルクのボトルラテ・SNS強</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
@@ -708,7 +710,7 @@
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>自家シロップ会社の旗艦。抹茶を材料使用。窓口明確</t>
+          <t>自家シロップ会社の旗艦・窓口明確</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
@@ -753,7 +755,7 @@
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>現在Uji（Yamasan）を外部調達→切替/比較提案の余地</t>
+          <t>Uji外部調達→切替/比較の余地</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
@@ -802,7 +804,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Honolulu随一の抹茶専門独立店。Japan直送＝品質志向、比較提案で</t>
+          <t>抹茶専門独立店・品質志向</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
@@ -847,7 +849,7 @@
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>地元コーヒー大手。抹茶も提供。多店舗＝数量見込み</t>
+          <t>地元コーヒー大手・多店舗で数量見込み</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
@@ -858,7 +860,455 @@
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>※ハワイは価格USD建て・米国内発が現実的。連絡先/店舗は変動→送信前に各IG/公式サイトのContactで最終確認を。メール直取得はサイト制限のため未完（DM/フォームが確実）。</t>
+          <t>※価格USD建て・米国内発が現実的。連絡先/店舗は変動→送信前に各IG/公式サイトのContactで最終確認を。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Fit / Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Area / Outlets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tel</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Priority note</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Contacted (date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Cowrie Coffee</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>324 Kapahulu Ave, Honolulu ／ Aiea ／ farmers markets</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>@cowriecoffee</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>cowriecoffee.square.site</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ヘルス志向の島焙煎・抹茶提供。独立系＝好機</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Cooke Street Market</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>725 Kapiolani Blvd（Kaka'ako）</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>@cookestreetmarket</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>csmhawaii.com</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>名物ストロベリー抹茶ラテ・人気店</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Morning Glass Coffee</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2955 E Manoa Rd（Manoa）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>@morningglasscoffee</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>morningglasscoffee.square.site</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>老舗ネイバーフッド・抹茶ソーダ等</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Aloha Matcha Hawaii</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>B寄り｜Matcha specialist</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Kaka'ako／Ala Moana ほかポップアップ</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ（DM）</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>@aloha.matcha.hi</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>抹茶＆ほうじ茶専門（自社調達）→競合寄りだが対話価値</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Pua Blooms</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent (pop-up)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kaka'ako（ポップアップ）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>点て立て抹茶・小規模だが感度高</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Kai Coffee Hawaii</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent (multi-outlet)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Waikiki 多店舗</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>@kaicoffeehawaii</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>kaicoffeehawaii.com</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>多店舗＝数量見込み。抹茶提供を要確認</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ARS Cafe</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>3116 Monsarrat Ave（Diamond Head）</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>@arscafe</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>ジェラート＋コーヒー。抹茶提供を要確認</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Dean &amp; DeLuca Hawaii</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>低優先｜準チェーン</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Ritz-Carlton Residences, Waikiki</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>@deandelucahawaii（要確認）</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>高級・準チェーン。抹茶提供あり・優先度低め</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>※追加候補。抹茶提供の有無・連絡先は送信前に各IG/サイトで要確認。Cowrie/Cooke Street/Morning Glass は独立系で抹茶確認済み＝A級で送付可。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 6 more Oahu café candidates (The Curb, Cha to Gelato Zen, Arvo, etc.)
Extend the Hawaii list and Excel Candidates sheet with The Curb Kaimuki,
Cha to Gelato Zen, Arvo Cafe, DEVOS Hawaii, Morning Brew Hawaii, and Lotus
Cafe, with IG/area from web research (matcha service flagged to verify
where not confirmed).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX28XCL3v6f7LuJT98rxVZ
</commit_message>
<xml_diff>
--- a/07_markets/us/HI_cafe_priority_A.xlsx
+++ b/07_markets/us/HI_cafe_priority_A.xlsx
@@ -876,7 +876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1305,8 +1305,262 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>The Curb Kaimuki</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Kaimuki, Honolulu</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>@thecurbkaimuki</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>スペシャルティ珈琲・パンダン抹茶ラテ等・独立系</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Cha to Gelato Zen</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜和テイスト</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>744 Kapahulu Ave, Honolulu</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>@cha_to_gelato_zen</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>抹茶＆ジェラート・点て立て抹茶</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Arvo Cafe</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent (multi)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Kaka'ako（Paiko）／Waikiki（Surfjack）</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>@a_r_v_o ／ @arvo_surfjack</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>arvocafe.com</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>映えるブランチカフェ・多店舗・抹茶提供</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>DEVOS Hawaiʻi</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Matcha pop-up</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ʻEwa（ポップアップ）</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>要確認（devos系）</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>新興の抹茶ポップアップ・感度高・小規模</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Morning Brew Hawaii</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent (multi)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Kailua／Kaka'ako 多店舗</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>@morningbrewhawaii</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>morningbrewhawaii.com</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>地元珈琲チェーン・多店舗＝数量・抹茶提供を要確認</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Lotus Cafe</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>A候補｜Independent</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Kaimuki, Honolulu</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>@lotuskaimuki</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>ネイバーフッドカフェ・抹茶提供を要確認</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>※追加候補。抹茶提供の有無・連絡先は送信前に各IG/サイトで要確認。Cowrie/Cooke Street/Morning Glass は独立系で抹茶確認済み＝A級で送付可。</t>
         </is>

</xml_diff>

<commit_message>
Expand Hawaii list to neighbor islands (Maui, Kauai, Big Island)
Add ~10 café prospects per neighbor island with area/IG from web research
(matcha and IG flagged to verify for coffee-first spots), in both the
Markdown list and new per-island Excel sheets. Multi-outlet chains noted as
higher priority.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX28XCL3v6f7LuJT98rxVZ
</commit_message>
<xml_diff>
--- a/07_markets/us/HI_cafe_priority_A.xlsx
+++ b/07_markets/us/HI_cafe_priority_A.xlsx
@@ -9,10 +9,16 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Priority A" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maui" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kauai" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Big Island" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Priority A'!$A$1:$M$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Candidates'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Maui'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Kauai'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Big Island'!$A$1:$M$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1570,4 +1576,1646 @@
   <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Fit / Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Area / Outlets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tel</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Priority note</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Contacted (date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Maui Matcha</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Matcha specialist</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Lahaina（Westin Nanea）／Wailea</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>@mauimatcha</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>抹茶専門・organic ceremonial。一部店舗休業情報→営業要確認</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Akamai Coffee Co.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Independent (multi)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kihei／Wailea／Kahului</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>@akamaicoffee</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>akamaicoffee.com</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>100%マウイ珈琲・抹茶ラテ提供</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Choice Health Bar</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Independent/health</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Ka'anapali／Paia</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>@choicehealthbar</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>choicehealthbar.com</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>アイス抹茶（Maui Matcha使用）</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>M4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Sip Me Maui</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Makawao（Baldwin Ave）</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>@sipmemaui（要確認）</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>アップカントリー定番・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>M5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Wailuku Coffee Company</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Wailuku（Market St）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>@wailukucoffeeco（要確認）</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>家族経営・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Crema Maui (at Marlow)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Pukalani</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>モダン珈琲・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>M7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Paia Bay Coffee</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Paia</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>@paiabaycoffee（要確認）</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>ビーチ隣接・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>M8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Anthony's Coffee Co.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Paia</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>@anthonyscoffeeco（要確認）</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>老舗ロースター・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>M9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Maui Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Kahului</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>@mauicoffeeroasters（要確認）</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>ロースター・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Espresso Mafia</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Makawao</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>抹茶ラテ提供</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>※マウイ候補。IG・抹茶提供は要確認。多店舗のAkamaiは数量見込みで優先度高め。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Fit / Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Area / Outlets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tel</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Priority note</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Contacted (date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Java Kai</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Independent (multi)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kapaa／Hanalei／Poipu／Princeville／Lihue</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>@javakai</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>javakai.com</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ストロベリー抹茶等・多店舗＝数量</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Little Fish Coffee</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Poipu（・Kapaa）</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>@littlefishcoffee</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>littlefishcoffee.com</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>南岸人気・抹茶</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Kalaheo Café &amp; Coffee Co.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Kalaheo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>@kalaheocoffee（要確認）</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>kalaheo.com</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>ラベンダー抹茶</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>K4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Small Town Coffee</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Kapaa</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>@smalltowncoffeeco（要確認）</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Kapaaの人気店</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Hanalei Bread Company</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Hanalei</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>@hanaleibread（要確認）</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>マンゴー抹茶（季節）</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Wishing Well</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Hanalei</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>@wishingwellshaveice（要確認）</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>アイス抹茶「Lili's Fav」</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>K7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The Spot North Shore</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Princeville</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>北岸ブランチ・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>K8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Kauai Coffee Company</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Independent (大)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Kalaheo</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>@kauaicoffeeco</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>kauaicoffee.com</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>大手農園カフェ・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>K9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ha Coffee Bar</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Lihue</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>@hacoffeebar（要確認）</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Lihue人気カフェ・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>K10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Trilogy Coffee</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Kapaa</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>@trilogycoffeekauai（要確認）</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>※カウアイ候補。IG・抹茶提供は要確認。多店舗のJava Kaiは数量見込みで優先度高め。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Café</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Fit / Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Area / Outlets</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tel</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Priority note</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Contacted (date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Kona Coffee &amp; Tea</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona（Palani Rd）</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>@konacoffeeandtea</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>konacoffeeandtea.com</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>農園カフェ・tea扱い・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Journey Cafe Big Island</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>@journeycafebigisland（要確認）</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>journeycafebigisland.com</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>アイス抹茶ラテ提供</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Big Island Coffee Roasters</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Hilo／Hakalau</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>@bigislandcoffeeroasters</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>bigislandcoffeeroasters.com</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>抹茶ラテ提供</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Hilo Coffee Mill</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Mountain View／Hilo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>@hilocoffeemill（要確認）</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>hilocoffeemill.com</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Kope Lani</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona（Kailua Bay）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>アイスラテ人気・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Waimea Coffee Company</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Waimea</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>@waimeacoffeecompany（要確認）</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>町の定番・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Papa Kona (ex-Daylight Mind)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>眺望カフェ・抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Kona Haven Coffee</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>@konahavencoffee（要確認）</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>H9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Basik Cafe</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>@basikacai（要確認）</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>açaí＋抹茶ボウル・要確認</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Sirius Coffee Connection</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Independent</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Kailua-Kona</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>要問合せ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>要確認</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>抹茶要確認</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>※ハワイ島候補。IG・抹茶提供は要確認。多店舗のKona Coffee &amp; Teaは数量見込みで優先度高め。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>